<commit_message>
progress: 27 village workbooks (randomwalk-TRX50-WS 2026-10-09T12:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -866,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -873,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B1, 1B2, 2A1A, 2A1B, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -880,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -887,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -894,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -901,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E1, 2E2, 3A, 3B, 3C, 3D, 4A, 4B, 5A1, 5A2, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -908,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -915,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -922,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -929,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -936,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -943,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -950,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -957,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -964,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1A1A1A1, 1A1B, 1A1C, 1A2, 1B, 1C, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -971,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C1, 1C2, 1D, 1E, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -978,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C1, 2C2, 2D, 2E1A, 2E1B, 2E2A, 2E2B, 2E2C, 3A, 3B1, 3B2, 3B3, 3B4, 3C1A, 3C1B, 3C1C, 3C1D, 3C1E, 3C2, 3C3, 3D1, 3D2, 3D3</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -985,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -992,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -999,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1C, 2A, 2B10, 2B11, 2B12, 2B1A, 2B1B, 2B2A, 2B2B, 2B3, 2B4A, 2B4B, 2B5, 2B6, 2B7, 2B8, 2B9, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1006,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1013,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1020,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1027,11 +1142,21 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
           <t>153</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2, 1B, 2A, 2B, 3, 4, 5, 6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 27 village workbooks (rw-rtx-3070 2026-10-09T15:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -1514,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1521,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C1, 3C2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1528,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1535,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1542,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 3</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1549,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 1D, 1E, 2, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B1, 6B2, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1556,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1563,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1570,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1577,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B, 3A1, 3A2, 3A3, 3A4, 3B, 3C1, 3C2, 3D1, 3D2, 3E, 3F1, 3F2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1584,6 +1634,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A1, 2A2, 2A3, 2B1, 2B2A1, 2B2B, 2B2C, 2B3A, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1591,6 +1646,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2A, 3A2B, 3B1A, 3B1B, 4A, 4B1, 4B2, 4B3</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1598,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 1C, 1D, 1E, 2A1, 2A2A, 2A2B, 2A2C, 2B1A1, 2B1A2, 2B1B, 2B2A, 2B2B, 2B2D</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1605,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1612,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1619,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1626,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B, 2B2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1633,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1640,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1647,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1A1, 1A10, 1A11, 1A12, 1A13, 1A14, 1A15A, 1A15B, 1A16, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9A, 1B1, 1B2, 1C, 1D, 2A, 2B1A, 2B1B1, 2B1B2, 2B1B3, 2B2, 2C1, 2C2, 2D1, 2D2, 2E, 2F, 2G, 2H, 3</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1654,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1661,6 +1766,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1O, 1P, 2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1668,6 +1778,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1675,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1C1, 1C2, 1C3, 2A, 2B1A, 2B1B, 2B1C1A1, 2B1C1B, 2B1C2, 2B1C3, 2B1C4, 2B1C5A1, 2B1C5B, 2B1C6, 2B2, 2C, 2D, 2E, 3, 4A1, 4A2, 4B, 4C1, 4C2A1, 4C2A2, 4C2B, 4C3A, 4C3B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1682,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1689,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1696,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1703,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1710,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1717,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1724,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1731,6 +1886,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 2, 32, 3A1A1A, 3A1A2, 3A1B, 3A2, 3B, 3C1, 3C2, 3D, 3E1, 3E2, 3F, 3G, 3H, 3I</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1738,6 +1898,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1745,6 +1910,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1752,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1759,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1766,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3A1, 3A2A, 3A2B, 3A3, 3A4A, 3A4B, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1773,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1780,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1787,6 +1982,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1794,6 +1994,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1801,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1808,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1815,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1822,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A1, 5B, 5C, 6A, 6B1, 6B2, 7, 8A, 8B, 8C, 8D, 8E, 8F, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1829,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1836,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1843,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1850,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1857,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A1, 4A2, 4A3, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1864,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A1D, 1A1E, 1A1F, 1A1G, 1A1H, 1A1I, 1A1J, 1A2, 1B, 1C1, 1C2, 1C3, 1C4, 1C5, 1C6, 1C7, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1871,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1878,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1885,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1892,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1899,6 +2174,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1906,6 +2186,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1913,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B, 1C, 1D, 2A, 2B, 2C, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1920,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1927,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1934,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1941,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2A, 2B1, 2B2A, 2B2B, 2B2C</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1948,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1955,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 3A, 3B, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -1962,6 +2282,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -1969,6 +2294,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -1976,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -1983,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 6, 7A1A, 7A1B, 7A2, 7B, 8A1A, 8A1B, 8A2, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -1990,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1A, 1B</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -1997,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2004,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2011,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2018,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2025,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2A1A1A1, 2A2B, 2A2C, 2A2D, 2A2E, 2A2F, 2A2G, 2A2H, 2A2J, 2B, 2C, 2D1, 2D2, 2D3, 2D4, 2E, 2F, 3A, 3B, 4A1A, 4A1B, 4A2, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2032,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2039,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2046,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B1, 2B2A1, 2B2B, 2B2C, 2C1A, 2C1B, 2C1C, 2C2, 2D1A1, 2D1B, 2D1C, 2D2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2053,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2060,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C1A1A, 1C1B, 1C1C, 1C1D, 1C2, 1D, 2A1A, 2A1A2, 2A1B, 2A2, 2B1, 2B2, 2B3, 2B4, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2067,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2074,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2081,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2088,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2095,6 +2510,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2102,6 +2522,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2109,6 +2534,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2116,6 +2546,11 @@
           <t>258A</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2123,6 +2558,11 @@
           <t>258B</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2130,6 +2570,11 @@
           <t>259A</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>A1, A2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2137,6 +2582,11 @@
           <t>259B</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>7, B1A, B1B, B2A1A1, B2A1B1, B2A1B2, B2A2, B2B, B3, B4A, B4B, B4C, B5A, B5B, B6</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2144,6 +2594,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4A, 4B, 5A, 5B1, 5B2, 6A, 6B, 6C, 7A, 7B, 8A, 8B, 8C1, 8C2</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2151,6 +2606,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2158,6 +2618,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2165,6 +2630,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2172,6 +2642,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 3F, 4A, 4B1, 4B2, 4B3, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2179,6 +2654,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2186,6 +2666,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C1, 1A1C2, 1A2, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2193,6 +2678,11 @@
           <t>266A</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3A3, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2200,6 +2690,11 @@
           <t>266B</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2207,6 +2702,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B, 3, 4A1, 4A2, 4A3, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2214,6 +2714,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2221,6 +2726,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1A, 1C1B1, 1C1B2, 1C2A, 1C2B, 2, 3A, 3B, 3B2, 3B3, 3B4, 3B5, 3B6</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2228,6 +2738,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2235,11 +2750,21 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
           <t>271</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 29 village workbooks (rw-rtx-3070 2026-10-09T15:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -2774,6 +2774,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2781,6 +2786,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2788,6 +2798,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1B4, 2A, 2B1, 2B2, 3A, 3B, 3C, 3D, 3E, 4A1A, 4A1B, 4A1C, 4A1D1, 4A2A, 4A2B1, 4A2B2A, 4A2B2B, 4A2B3, 4B1, 4B2A1, 4B2A2, 4B2B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2795,6 +2810,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2802,6 +2822,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2809,6 +2834,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2816,6 +2846,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2A, 2A2B, 2A3, 2B1, 2B10, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 2B9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2823,6 +2858,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2830,6 +2870,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2837,6 +2882,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2844,6 +2894,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1A, 3A1B, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2851,6 +2906,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2858,6 +2918,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2865,6 +2930,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1A, 2A1B, 2A2A, 2A2B, 2B1, 2B2, 2C1A1, 2C1B, 2C2, 3, 4A1A1, 4A1B, 4A2, 4B, 5A, 5B, 5C, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2872,6 +2942,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2879,6 +2954,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 1C1, 1C2A, 1C2B, 1D, 1E1, 1E2, 2A1A1, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2A8, 2A9, 2B, 2C, 2D, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2886,6 +2966,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2893,6 +2978,11 @@
           <t>288A</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2900,6 +2990,11 @@
           <t>288B</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1A, 1B, B2, B3</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2907,6 +3002,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2914,6 +3014,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2921,6 +3026,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2928,6 +3038,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3A, 2A3B1, 2A3B2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2935,6 +3050,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2942,6 +3062,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2949,6 +3074,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2956,6 +3086,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2963,6 +3098,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2970,6 +3110,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2977,6 +3122,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2984,6 +3134,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1C</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2991,6 +3146,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2998,6 +3158,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -3005,6 +3170,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -3012,6 +3182,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3019,6 +3194,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3026,6 +3206,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3033,6 +3218,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3040,6 +3230,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C1, 1A1C2, 1A2, 1B, 1C, 1D, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3047,6 +3242,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4A1, 4A2, 4B1, 4B2, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3054,6 +3254,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3061,6 +3266,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 4B3, 4B4, 4B5, 5A, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3068,6 +3278,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3075,6 +3290,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3082,6 +3302,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3089,6 +3314,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3096,6 +3326,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1A2, 1A2, 1A3, 1A4, 1B, 1C1, 1C2, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3103,6 +3338,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A1A1A1, 1B, 1C, 1D, 1E, 1F, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A2A, 2A1A2B1, 2A1B, 2A2A, 2A2A2, 2B1A1A1, 2B1B1, 2B2A1, 2B2A2, 2C, 2D1A1, 2D2A, 2D2B, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3110,6 +3350,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B1, 1A1B2, 1A2, 1A3, 1A4, 1A5, 1B1A1A1A1, 1B1A2, 1B2, 1B3, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A1A, 2A1B, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2B1A1A, 2B1B, 2B2, 2C, 2D, 2E, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3117,6 +3362,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3124,6 +3374,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3131,6 +3386,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3138,6 +3398,11 @@
           <t>318A</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3145,6 +3410,11 @@
           <t>318B</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3152,6 +3422,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3159,6 +3434,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3166,6 +3446,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3173,6 +3458,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3180,6 +3470,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3187,6 +3482,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3194,6 +3494,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3201,6 +3506,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3A, 1B3B, 1B4A, 1B4B, 1B5A, 1B5B, 1B5C, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3208,6 +3518,11 @@
           <t>326A</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3215,6 +3530,11 @@
           <t>326B</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3222,6 +3542,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 1C, 1D, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3229,6 +3554,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 3A1A, 3A1B, 3A1C1, 3A1C2, 3A2, 3A3, 3B, 3C1, 3C2A1, 3C2A2A, 3C2A3, 3C2B1, 3C2B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3236,6 +3566,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3243,6 +3578,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3250,6 +3590,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3257,6 +3602,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B, 1C1A1A, 1C1A1B1, 1C1A1B2, 1C1A1C1, 1C1A1C2, 1C1A1D, 1C1A1E, 1C1A2, 1C1B1, 1C1B2, 1C1C1A, 1C1C1B3, 1C1C1B4, 1C1C1B5A, 1C1C1B6, 1C1CB1, 1C1CB2, 1C2A1, 1C2A2, 1C2B, 1D1, 1D2, 1E1, 1E2, 2, 3A1, 3A2, 3A3, 3B1, 3B2, 3B3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3264,6 +3614,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3271,6 +3626,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3278,6 +3638,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3285,6 +3650,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3292,6 +3662,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3299,6 +3674,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C1, 10C2, 11A, 11B, 11C, 12A, 12B, 13, 14A, 14B, 15, 1A, 1B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3306,6 +3686,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B1, 1B2, 1B3, 1C1A, 1C1B, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3313,6 +3698,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3320,6 +3710,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B1A1, 1B1A2, 1B1A3, 1B1B, 1B1C, 1B1D, 1B2A, 1B2B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3327,6 +3722,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3334,6 +3734,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1A4A, 1A4B, 1A4C, 1B1, 1B2, 2A1A, 2A1A1, 2A1B, 2A3A1A, 2A3A1B, 2A3A2, 2A3B, 2B1, 2B2A, 2B2B1, 3A, 3B1, 3B2, 3C, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3341,6 +3746,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3348,6 +3758,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3355,6 +3770,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A2, 2A3, 2A4, 2B, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3B1A, 3B1B, 3B1C, 3B1D, 3B1E, 3B1F, 3B1G, 3B1H, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3362,6 +3782,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3369,6 +3794,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 3A1A1, 3A1A2, 3A1B, 3A2, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3376,6 +3806,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2A1, 2A2B, 2A2C, 2A2D, 2A2E, 2A2F, 2B1, 2B2, 2B3, 2B4, 2B5, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3383,6 +3818,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A1, 4A2A, 4A2B, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3390,6 +3830,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4A1, 1B4A2, 1B4B, 2A, 2B1, 2B2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3397,6 +3842,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3404,6 +3854,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3411,6 +3866,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3418,6 +3878,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A1, 2B1B, 2B2, 2B3, 2B4, 2C1, 2C2, 2C2B, 3A1A1, 3A1A2, 3A1B1, 3A1B2, 3A1B3, 3A1B4, 3A1B5, 3A2, 3B, 4A1, 4A2, 4A3A, 4A3B, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3425,6 +3890,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3432,6 +3902,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3439,6 +3914,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A1, 4A2, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3446,6 +3926,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1B4, 1C1, 1C2, 1C3, 1C4, 1C5, 1C6, 1C7, 1C8A1, 1C8B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3453,6 +3938,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3460,6 +3950,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3467,6 +3962,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3474,6 +3974,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7A1, 7A2, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3481,6 +3986,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 2B3, 2B4A, 2B4B, 2B5, 2B6, 2B7, 2B8, 2B9, 3, 4A1, 4A2, 4B, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3488,11 +3998,21 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
           <t>362</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B1A1, 2B1A2, 2B1B, 2B1C1, 2B1C2, 2B1D1, 2B1D2, 2B1D3, 2B1E1, 2B1E2, 2B1E3, 2B1E4, 2B1E5, 2B1E6, 2B1E7, 2B2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 30 village workbooks (rw-rtx-3070 2026-10-09T15:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -4022,6 +4022,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -4029,6 +4034,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -4036,6 +4046,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -4043,6 +4058,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -4050,6 +4070,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -4057,6 +4082,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -4064,6 +4094,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -4071,6 +4106,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -4078,6 +4118,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -4085,6 +4130,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -4092,6 +4142,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -4099,6 +4154,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B1, 3B2, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4106,6 +4166,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4113,6 +4178,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4120,6 +4190,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4127,6 +4202,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4134,6 +4214,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4141,6 +4226,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4148,6 +4238,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4155,6 +4250,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4162,6 +4262,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B1, 1B1B2, 1B1C, 1B1D1, 1B1D2, 1B2, 1B3, 1C, 1D, 1E, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4169,6 +4274,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2A, 2B2B, 2B2C, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4176,6 +4286,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4183,6 +4298,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4190,6 +4310,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4197,6 +4322,11 @@
           <t>386</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4204,6 +4334,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4211,6 +4346,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4218,6 +4358,11 @@
           <t>389</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4225,6 +4370,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4232,6 +4382,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4239,6 +4394,11 @@
           <t>391</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4246,6 +4406,11 @@
           <t>392</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4253,6 +4418,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4260,6 +4430,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A2A, 2A2B, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4267,6 +4442,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4274,6 +4454,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4281,6 +4466,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4288,6 +4478,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4295,6 +4490,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4302,6 +4502,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4309,6 +4514,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4316,6 +4526,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4323,6 +4538,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4330,6 +4550,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4337,6 +4562,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4344,6 +4574,11 @@
           <t>404</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4351,6 +4586,11 @@
           <t>405</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4358,6 +4598,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4365,6 +4610,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4372,6 +4622,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4379,6 +4634,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4386,6 +4646,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4393,6 +4658,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B1C, 1B2, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4400,6 +4670,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4407,6 +4682,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4414,6 +4694,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4421,6 +4706,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4428,6 +4718,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4435,6 +4730,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A1, 2A1A2, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4442,6 +4742,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2A, 2A1, 2A2, 2B1, 2B2, 2B3, 3</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4449,6 +4754,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4456,6 +4766,11 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2A, 1C2B, 2A1, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4463,6 +4778,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4470,6 +4790,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4477,6 +4802,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4484,6 +4814,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4491,6 +4826,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4498,6 +4838,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4505,6 +4850,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4512,6 +4862,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4519,6 +4874,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4526,6 +4886,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4533,6 +4898,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4540,6 +4910,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4547,6 +4922,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4554,6 +4934,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4561,6 +4946,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4568,6 +4958,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4575,6 +4970,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4582,6 +4982,11 @@
           <t>435</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4589,6 +4994,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4596,6 +5006,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2, 3, 4A1, 4A2, 4B1, 4B2, 4C1, 4C2, 4D1, 4D2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4603,6 +5018,11 @@
           <t>438</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4610,6 +5030,11 @@
           <t>439</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4617,6 +5042,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4624,6 +5054,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4631,6 +5066,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4638,6 +5078,11 @@
           <t>442</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -4645,6 +5090,11 @@
           <t>443</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -4652,6 +5102,11 @@
           <t>444</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -4659,6 +5114,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -4666,6 +5126,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -4673,6 +5138,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -4680,6 +5150,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -4687,6 +5162,11 @@
           <t>449</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -4694,6 +5174,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3A1, 3A2, 3B, 4A1, 4A2, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -4701,6 +5186,11 @@
           <t>450</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -4708,6 +5198,11 @@
           <t>451</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -4715,6 +5210,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -4722,6 +5222,11 @@
           <t>453</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -4729,6 +5234,11 @@
           <t>454</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -4736,11 +5246,21 @@
           <t>455</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
           <t>456</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 32 village workbooks (rw-rtx-3070 2026-10-09T15:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -5270,6 +5270,11 @@
           <t>457</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1B, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1B1A1, 1B1B, 1B1C, 1B1D, 1B2A1, 1B2B, 1B2C, 1B2D, 20, 21, 22, 23, 24, 25, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3A1A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3J, 3K, 4A10, 4A1A1, 4A1B, 4A1C, 4A2, 4A3, 4A4, 4A5, 4A6, 4A7, 4A8, 4A9, 4B1A1A1A1A, 4B1B, 4B2, 5A1, 5A2, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -5277,6 +5282,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1B, 1A1C, 1A2A1A, 1A2A2, 1A2B, 1A2C, 1A2D, 1A2E, 1A2F, 1A2G, 1B1A1A, 1B1B, 1B1C, 1B1D, 1B2A1A1, 1B2B, 1B2C, 1B2D, 1B2E, 1B2F, 1B2G, 1B2H, 1C1A1A, 1C1B, 1C2A1A1A, 1C2B, 20, 21, 22, 23, 24, 26, 27, 2A1A1A1A, 2A1B, 2A1C, 2A2, 2B, 3A1A1A, 3A1B, 3A2, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -5284,6 +5294,11 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -5291,6 +5306,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5298,6 +5318,11 @@
           <t>460</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 1A2, 1A3, 1A4, 1A5, 1B1, 1B2, 1B3, 2A1A, 2A1B, 2A1C, 2A2, 2B1A, 2B1B, 2B2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5305,6 +5330,11 @@
           <t>461</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5312,6 +5342,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5319,6 +5354,11 @@
           <t>463</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -5326,6 +5366,11 @@
           <t>464A</t>
         </is>
       </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -5333,6 +5378,11 @@
           <t>464B</t>
         </is>
       </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A2C, 1A3, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -5340,6 +5390,11 @@
           <t>465A</t>
         </is>
       </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B1, 2B2, 2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -5347,6 +5402,11 @@
           <t>465B</t>
         </is>
       </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1, 1A2, 1A3, 1B, 2, 3A, 3B1, 3B1B, 3B2, 4A1, 4A2, 4B, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -5354,6 +5414,11 @@
           <t>466</t>
         </is>
       </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -5361,6 +5426,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -5368,6 +5438,11 @@
           <t>468A</t>
         </is>
       </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -5375,6 +5450,11 @@
           <t>468B</t>
         </is>
       </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2B, 2B1, 2B2, 3, 4A, 4B, 4C, 5</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -5382,6 +5462,11 @@
           <t>469</t>
         </is>
       </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -5389,6 +5474,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 2A, 2B1, 2B2, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -5396,6 +5486,11 @@
           <t>470</t>
         </is>
       </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -5403,6 +5498,11 @@
           <t>471</t>
         </is>
       </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2A1, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -5410,6 +5510,11 @@
           <t>472</t>
         </is>
       </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -5417,6 +5522,11 @@
           <t>473</t>
         </is>
       </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -5424,6 +5534,11 @@
           <t>474</t>
         </is>
       </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -5431,6 +5546,11 @@
           <t>475</t>
         </is>
       </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -5438,6 +5558,11 @@
           <t>476</t>
         </is>
       </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -5445,6 +5570,11 @@
           <t>477</t>
         </is>
       </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -5452,6 +5582,11 @@
           <t>478</t>
         </is>
       </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -5459,6 +5594,11 @@
           <t>479</t>
         </is>
       </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -5466,6 +5606,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -5473,6 +5618,11 @@
           <t>480</t>
         </is>
       </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -5480,6 +5630,11 @@
           <t>481</t>
         </is>
       </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -5487,6 +5642,11 @@
           <t>482</t>
         </is>
       </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1A, 2B1B, 2B1C, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -5494,6 +5654,11 @@
           <t>483</t>
         </is>
       </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -5501,6 +5666,11 @@
           <t>484</t>
         </is>
       </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -5508,6 +5678,11 @@
           <t>485</t>
         </is>
       </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -5515,6 +5690,11 @@
           <t>486</t>
         </is>
       </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A1C, 1A1D, 1A2, 1A3, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -5522,6 +5702,11 @@
           <t>487</t>
         </is>
       </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -5529,6 +5714,11 @@
           <t>488</t>
         </is>
       </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -5536,6 +5726,11 @@
           <t>489</t>
         </is>
       </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -5543,6 +5738,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -5550,6 +5750,11 @@
           <t>490</t>
         </is>
       </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E1, 1E2, 2A, 2B, 2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -5557,6 +5762,11 @@
           <t>491</t>
         </is>
       </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -5564,6 +5774,11 @@
           <t>492</t>
         </is>
       </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -5571,6 +5786,11 @@
           <t>493</t>
         </is>
       </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -5578,6 +5798,11 @@
           <t>494</t>
         </is>
       </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -5585,6 +5810,11 @@
           <t>495</t>
         </is>
       </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -5592,6 +5822,11 @@
           <t>496</t>
         </is>
       </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -5599,6 +5834,11 @@
           <t>497</t>
         </is>
       </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -5606,6 +5846,11 @@
           <t>498</t>
         </is>
       </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -5613,6 +5858,11 @@
           <t>499</t>
         </is>
       </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -5620,6 +5870,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 2B4, 3A, 3B1A, 3B1B, 3B1C, 3B2, 3B3, 3B4, 4</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -5627,6 +5882,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -5634,6 +5894,11 @@
           <t>501</t>
         </is>
       </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2, 3A, 3B1, 3B2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -5641,6 +5906,11 @@
           <t>502</t>
         </is>
       </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -5648,6 +5918,11 @@
           <t>503</t>
         </is>
       </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -5655,6 +5930,11 @@
           <t>504</t>
         </is>
       </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -5662,6 +5942,11 @@
           <t>505</t>
         </is>
       </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -5669,11 +5954,21 @@
           <t>506</t>
         </is>
       </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
           <t>507</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3A1, 2A3A2, 2A3B, 2B, 3, 4A, 4B1, 4B2, 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 35 village workbooks (rw-rtx-3070 2026-10-09T22:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -8330,6 +8330,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -8337,6 +8342,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
@@ -8344,11 +8354,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 52 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -1166,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1A4, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1173,6 +1178,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1180,6 +1190,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A3A, 1A3B, 1B1A, 1B1B, 1B2, 2, 3A, 3B, 4A, 4B1, 4B2, 4C1A, 4C1B, 4C2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1187,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1A, 1A2, 1A3, 1A4, 1B1, 1B2, 2A1, 2A2, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1194,11 +1214,21 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
           <t>159</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 1B3, 1B4, 2A, 2B, 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 52 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -1238,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1245,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6A, 6B1, 6B2, 7A1, 7A2, 7B, 7C, 7D, 7E, 7F, 7G</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1252,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1C1, 1C2, 1C3, 1C4A, 1C4B, 1C4C, 1D, 2A1, 2A2, 2B, 2C, 3A1, 3A2A, 3A2B, 3A2C, 3B1, 3B2A, 3B2B, 3B2C, 4, 5A1, 5A2, 5A3, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1259,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6A, 6B, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1266,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1273,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A1A, 1A2B, 1A3, 1A4A, 1A4B, 1A4C, 1A4D, 1A4E, 1A4F1, 1B1, 1B2, 1B3, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1280,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1287,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1294,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1301,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1308,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1315,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1A4, 1B1, 1B2, 1C1, 1C2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1322,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1329,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1336,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1343,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1350,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1357,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1364,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1371,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1378,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1385,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1392,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1399,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1406,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C1, 3C2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1413,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1420,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1427,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 3</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1434,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 1D, 1E, 2, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B1, 6B2, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1441,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1448,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1455,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1462,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B, 3A1, 3A2, 3A3, 3A4, 3B, 3C1, 3C2, 3D1, 3D2, 3E, 3F1, 3F2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1469,6 +1634,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A1, 2A2, 2A3, 2B1, 2B2A1, 2B2B, 2B2C, 2B3A, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1476,6 +1646,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2A, 3A2B, 3B1A, 3B1B, 4A, 4B1, 4B2, 4B3</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1483,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 1C, 1D, 1E, 2A1, 2A2A, 2A2B, 2A2C, 2B1A1, 2B1A2, 2B1B, 2B2A, 2B2B, 2B2D</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1490,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1497,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1504,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1511,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B, 2B2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1518,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1525,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1532,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1A1, 1A10, 1A11, 1A12, 1A13, 1A14, 1A15A, 1A15B, 1A16, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9A, 1B1, 1B2, 1C, 1D, 2A, 2B1A, 2B1B1, 2B1B2, 2B1B3, 2B2, 2C1, 2C2, 2D1, 2D2, 2E, 2F, 2G, 2H, 3</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1539,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1546,6 +1766,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1O, 1P, 2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1553,6 +1778,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1560,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1C1, 1C2, 1C3, 2A, 2B1A, 2B1B, 2B1C1A1, 2B1C1B, 2B1C2, 2B1C3, 2B1C4, 2B1C5A1, 2B1C5B, 2B1C6, 2B2, 2C, 2D, 2E, 3, 4A1, 4A2, 4B, 4C1, 4C2A1, 4C2A2, 4C2B, 4C3A, 4C3B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1567,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1574,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1581,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1588,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1595,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1602,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1609,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1616,6 +1886,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 2, 32, 3A1A1A, 3A1A2, 3A1B, 3A2, 3B, 3C1, 3C2, 3D, 3E1, 3E2, 3F, 3G, 3H, 3I</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1623,6 +1898,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1630,6 +1910,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1637,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1644,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1651,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3A1, 3A2A, 3A2B, 3A3, 3A4A, 3A4B, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1658,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1665,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1672,6 +1982,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1679,6 +1994,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1686,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1693,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1700,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1707,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A1, 5B, 5C, 6A, 6B1, 6B2, 7, 8A, 8B, 8C, 8D, 8E, 8F, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1714,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1721,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1728,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1735,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1742,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A1, 4A2, 4A3, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1749,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A1D, 1A1E, 1A1F, 1A1G, 1A1H, 1A1I, 1A1J, 1A2, 1B, 1C1, 1C2, 1C3, 1C4, 1C5, 1C6, 1C7, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1756,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1763,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1770,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1777,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1784,6 +2174,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1791,6 +2186,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1798,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B, 1C, 1D, 2A, 2B, 2C, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1805,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1812,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1819,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1826,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2A, 2B1, 2B2A, 2B2B, 2B2C</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1833,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1840,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 3A, 3B, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -1847,11 +2282,21 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
           <t>239</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 54 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -2306,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2313,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 6, 7A1A, 7A1B, 7A2, 7B, 8A1A, 8A1B, 8A2, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2320,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1A, 1B</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2327,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2334,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2341,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2348,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2355,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2A1A1A1, 2A2B, 2A2C, 2A2D, 2A2E, 2A2F, 2A2G, 2A2H, 2A2J, 2B, 2C, 2D1, 2D2, 2D3, 2D4, 2E, 2F, 3A, 3B, 4A1A, 4A1B, 4A2, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2362,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2369,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2376,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B1, 2B2A1, 2B2B, 2B2C, 2C1A, 2C1B, 2C1C, 2C2, 2D1A1, 2D1B, 2D1C, 2D2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2383,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2390,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C1A1A, 1C1B, 1C1C, 1C1D, 1C2, 1D, 2A1A, 2A1A2, 2A1B, 2A2, 2B1, 2B2, 2B3, 2B4, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2397,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2404,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2411,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2418,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2425,6 +2510,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2432,6 +2522,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2439,6 +2534,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2446,6 +2546,11 @@
           <t>258A</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2453,6 +2558,11 @@
           <t>258B</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2460,6 +2570,11 @@
           <t>259A</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>A1, A2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2467,6 +2582,11 @@
           <t>259B</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>7, B1A, B1B, B2A1A1, B2A1B1, B2A1B2, B2A2, B2B, B3, B4A, B4B, B4C, B5A, B5B, B6</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2474,6 +2594,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4A, 4B, 5A, 5B1, 5B2, 6A, 6B, 6C, 7A, 7B, 8A, 8B, 8C1, 8C2</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2481,6 +2606,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2488,6 +2618,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2495,6 +2630,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2502,6 +2642,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 3F, 4A, 4B1, 4B2, 4B3, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2509,6 +2654,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2516,6 +2666,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C1, 1A1C2, 1A2, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2523,6 +2678,11 @@
           <t>266A</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3A3, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2530,6 +2690,11 @@
           <t>266B</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2537,6 +2702,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B, 3, 4A1, 4A2, 4A3, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2544,6 +2714,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2551,6 +2726,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1A, 1C1B1, 1C1B2, 1C2A, 1C2B, 2, 3A, 3B, 3B2, 3B3, 3B4, 3B5, 3B6</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2558,6 +2738,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2565,6 +2750,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2572,6 +2762,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2579,6 +2774,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2586,6 +2786,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2593,6 +2798,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1B4, 2A, 2B1, 2B2, 3A, 3B, 3C, 3D, 3E, 4A1A, 4A1B, 4A1C, 4A1D1, 4A2A, 4A2B1, 4A2B2A, 4A2B2B, 4A2B3, 4B1, 4B2A1, 4B2A2, 4B2B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2600,6 +2810,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2607,6 +2822,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2614,6 +2834,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2621,6 +2846,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2A, 2A2B, 2A3, 2B1, 2B10, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 2B9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2628,6 +2858,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2635,6 +2870,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2642,6 +2882,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2649,6 +2894,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1A, 3A1B, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2656,6 +2906,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2663,6 +2918,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2670,6 +2930,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1A, 2A1B, 2A2A, 2A2B, 2B1, 2B2, 2C1A1, 2C1B, 2C2, 3, 4A1A1, 4A1B, 4A2, 4B, 5A, 5B, 5C, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2677,6 +2942,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2684,6 +2954,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 1C1, 1C2A, 1C2B, 1D, 1E1, 1E2, 2A1A1, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2A8, 2A9, 2B, 2C, 2D, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2691,6 +2966,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2698,6 +2978,11 @@
           <t>288A</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2705,6 +2990,11 @@
           <t>288B</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1A, 1B, B2, B3</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2712,6 +3002,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2719,6 +3014,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2726,6 +3026,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2733,6 +3038,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3A, 2A3B1, 2A3B2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2740,6 +3050,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2747,6 +3062,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2754,6 +3074,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2761,6 +3086,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2768,6 +3098,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2775,6 +3110,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2782,6 +3122,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2789,6 +3134,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1C</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2796,6 +3146,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2803,6 +3158,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2810,6 +3170,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2817,6 +3182,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2824,6 +3194,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2831,6 +3206,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2838,6 +3218,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -2845,6 +3230,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C1, 1A1C2, 1A2, 1B, 1C, 1D, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -2852,6 +3242,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4A1, 4A2, 4B1, 4B2, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -2859,6 +3254,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A1, 2A2, 2B1A, 2B1B, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -2866,6 +3266,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 4B3, 4B4, 4B5, 5A, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -2873,6 +3278,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -2880,6 +3290,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -2887,6 +3302,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -2894,6 +3314,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -2901,6 +3326,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1A2, 1A2, 1A3, 1A4, 1B, 1C1, 1C2, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -2908,6 +3338,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A1A1A1, 1B, 1C, 1D, 1E, 1F, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A2A, 2A1A2B1, 2A1B, 2A2A, 2A2A2, 2B1A1A1, 2B1B1, 2B2A1, 2B2A2, 2C, 2D1A1, 2D2A, 2D2B, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -2915,6 +3350,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B1, 1A1B2, 1A2, 1A3, 1A4, 1A5, 1B1A1A1A1, 1B1A2, 1B2, 1B3, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A1A, 2A1B, 2A2, 2A3, 2A4, 2A5, 2A6, 2A7, 2B1A1A, 2B1B, 2B2, 2C, 2D, 2E, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -2922,6 +3362,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -2929,6 +3374,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -2936,11 +3386,21 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
           <t>318A</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 55 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -3410,6 +3410,11 @@
           <t>318B</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3417,6 +3422,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3424,6 +3434,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3431,6 +3446,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3438,6 +3458,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3445,6 +3470,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3452,6 +3482,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3459,6 +3494,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3466,6 +3506,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3A, 1B3B, 1B4A, 1B4B, 1B5A, 1B5B, 1B5C, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3473,6 +3518,11 @@
           <t>326A</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3480,6 +3530,11 @@
           <t>326B</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3487,6 +3542,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 1C, 1D, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3494,6 +3554,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 3A1A, 3A1B, 3A1C1, 3A1C2, 3A2, 3A3, 3B, 3C1, 3C2A1, 3C2A2A, 3C2A3, 3C2B1, 3C2B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3501,6 +3566,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3508,6 +3578,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3515,6 +3590,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3522,6 +3602,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B, 1C1A1A, 1C1A1B1, 1C1A1B2, 1C1A1C1, 1C1A1C2, 1C1A1D, 1C1A1E, 1C1A2, 1C1B1, 1C1B2, 1C1C1A, 1C1C1B3, 1C1C1B4, 1C1C1B5A, 1C1C1B6, 1C1CB1, 1C1CB2, 1C2A1, 1C2A2, 1C2B, 1D1, 1D2, 1E1, 1E2, 2, 3A1, 3A2, 3A3, 3B1, 3B2, 3B3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3529,6 +3614,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3536,6 +3626,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3543,6 +3638,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3550,6 +3650,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3557,6 +3662,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3564,6 +3674,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C1, 10C2, 11A, 11B, 11C, 12A, 12B, 13, 14A, 14B, 15, 1A, 1B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3571,6 +3686,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1B1, 1B2, 1B3, 1C1A, 1C1B, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3578,6 +3698,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3585,6 +3710,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B1A1, 1B1A2, 1B1A3, 1B1B, 1B1C, 1B1D, 1B2A, 1B2B, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3592,6 +3722,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3599,6 +3734,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3, 1A4A, 1A4B, 1A4C, 1B1, 1B2, 2A1A, 2A1A1, 2A1B, 2A3A1A, 2A3A1B, 2A3A2, 2A3B, 2B1, 2B2A, 2B2B1, 3A, 3B1, 3B2, 3C, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3606,6 +3746,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3613,6 +3758,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3620,6 +3770,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A2, 2A3, 2A4, 2B, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3B1A, 3B1B, 3B1C, 3B1D, 3B1E, 3B1F, 3B1G, 3B1H, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3627,6 +3782,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3634,6 +3794,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 3A1A1, 3A1A2, 3A1B, 3A2, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3641,6 +3806,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2A1, 2A2B, 2A2C, 2A2D, 2A2E, 2A2F, 2B1, 2B2, 2B3, 2B4, 2B5, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3648,6 +3818,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A1, 4A2A, 4A2B, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3655,6 +3830,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4A1, 1B4A2, 1B4B, 2A, 2B1, 2B2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3662,6 +3842,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3669,6 +3854,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3676,6 +3866,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3683,6 +3878,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A1, 2B1B, 2B2, 2B3, 2B4, 2C1, 2C2, 2C2B, 3A1A1, 3A1A2, 3A1B1, 3A1B2, 3A1B3, 3A1B4, 3A1B5, 3A2, 3B, 4A1, 4A2, 4A3A, 4A3B, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3690,6 +3890,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3697,6 +3902,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3704,6 +3914,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A1, 4A2, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3711,6 +3926,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1B4, 1C1, 1C2, 1C3, 1C4, 1C5, 1C6, 1C7, 1C8A1, 1C8B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3718,6 +3938,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3725,6 +3950,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3732,6 +3962,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3739,6 +3974,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7A1, 7A2, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3746,6 +3986,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 2B3, 2B4A, 2B4B, 2B5, 2B6, 2B7, 2B8, 2B9, 3, 4A1, 4A2, 4B, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3753,6 +3998,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3760,6 +4010,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B1A1, 2B1A2, 2B1B, 2B1C1, 2B1C2, 2B1D1, 2B1D2, 2B1D3, 2B1E1, 2B1E2, 2B1E3, 2B1E4, 2B1E5, 2B1E6, 2B1E7, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3767,6 +4022,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3774,6 +4034,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3781,6 +4046,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3788,6 +4058,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3795,6 +4070,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3802,6 +4082,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3809,6 +4094,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3816,6 +4106,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3823,6 +4118,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3830,6 +4130,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3837,6 +4142,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -3844,6 +4154,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B1, 3B2, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -3851,6 +4166,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -3858,6 +4178,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -3865,6 +4190,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -3872,6 +4202,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -3879,6 +4214,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -3886,6 +4226,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -3893,6 +4238,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -3900,6 +4250,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -3907,6 +4262,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B1, 1B1B2, 1B1C, 1B1D1, 1B1D2, 1B2, 1B3, 1C, 1D, 1E, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -3914,6 +4274,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2A, 2B2B, 2B2C, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -3921,6 +4286,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -3928,6 +4298,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -3935,6 +4310,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -3942,6 +4322,11 @@
           <t>386</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -3949,6 +4334,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -3956,6 +4346,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -3963,6 +4358,11 @@
           <t>389</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -3970,6 +4370,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -3977,11 +4382,21 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
           <t>391</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 55 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -4406,6 +4406,11 @@
           <t>392</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4413,6 +4418,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4420,6 +4430,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A2A, 2A2B, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4427,6 +4442,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4434,6 +4454,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4441,6 +4466,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4448,6 +4478,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4455,6 +4490,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4462,6 +4502,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4469,6 +4514,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4476,6 +4526,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4483,6 +4538,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4490,6 +4550,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4497,6 +4562,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4504,6 +4574,11 @@
           <t>404</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4511,6 +4586,11 @@
           <t>405</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4518,6 +4598,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4525,6 +4610,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4532,6 +4622,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4539,6 +4634,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4546,6 +4646,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4553,6 +4658,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B1C, 1B2, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4560,6 +4670,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4567,6 +4682,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4574,6 +4694,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4581,6 +4706,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4588,6 +4718,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4595,6 +4730,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A1, 2A1A2, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4602,6 +4742,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2A, 2A1, 2A2, 2B1, 2B2, 2B3, 3</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4609,6 +4754,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4616,6 +4766,11 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2A, 1C2B, 2A1, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4623,6 +4778,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4630,6 +4790,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4637,6 +4802,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4644,6 +4814,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4651,6 +4826,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4658,6 +4838,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4665,6 +4850,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4672,6 +4862,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4679,6 +4874,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4686,6 +4886,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4693,6 +4898,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4700,6 +4910,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4707,6 +4922,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4714,6 +4934,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4721,6 +4946,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4728,6 +4958,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4735,6 +4970,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A1, 2A2, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4742,6 +4982,11 @@
           <t>435</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4749,6 +4994,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4756,6 +5006,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2, 3, 4A1, 4A2, 4B1, 4B2, 4C1, 4C2, 4D1, 4D2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4763,6 +5018,11 @@
           <t>438</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4770,6 +5030,11 @@
           <t>439</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4777,6 +5042,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4784,6 +5054,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4791,6 +5066,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4798,6 +5078,11 @@
           <t>442</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -4805,6 +5090,11 @@
           <t>443</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -4812,6 +5102,11 @@
           <t>444</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -4819,6 +5114,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -4826,6 +5126,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -4833,6 +5138,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -4840,6 +5150,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -4847,6 +5162,11 @@
           <t>449</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -4854,6 +5174,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3A1, 3A2, 3B, 4A1, 4A2, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -4861,6 +5186,11 @@
           <t>450</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -4868,6 +5198,11 @@
           <t>451</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -4875,6 +5210,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -4882,6 +5222,11 @@
           <t>453</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -4889,6 +5234,11 @@
           <t>454</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -4896,6 +5246,11 @@
           <t>455</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -4903,6 +5258,11 @@
           <t>456</t>
         </is>
       </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -4910,6 +5270,11 @@
           <t>457</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1B, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1B1A1, 1B1B, 1B1C, 1B1D, 1B2A1, 1B2B, 1B2C, 1B2D, 20, 21, 22, 23, 24, 25, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3A1A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3J, 3K, 4A10, 4A1A1, 4A1B, 4A1C, 4A2, 4A3, 4A4, 4A5, 4A6, 4A7, 4A8, 4A9, 4B1A1A1A1A, 4B1B, 4B2, 5A1, 5A2, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -4917,6 +5282,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1B, 1A1C, 1A2A1A, 1A2A2, 1A2B, 1A2C, 1A2D, 1A2E, 1A2F, 1A2G, 1B1A1A, 1B1B, 1B1C, 1B1D, 1B2A1A1, 1B2B, 1B2C, 1B2D, 1B2E, 1B2F, 1B2G, 1B2H, 1C1A1A, 1C1B, 1C2A1A1A, 1C2B, 20, 21, 22, 23, 24, 26, 27, 2A1A1A1A, 2A1B, 2A1C, 2A2, 2B, 3A1A1A, 3A1B, 3A2, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -4924,6 +5294,11 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -4931,6 +5306,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -4938,6 +5318,11 @@
           <t>460</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 1A2, 1A3, 1A4, 1A5, 1B1, 1B2, 1B3, 2A1A, 2A1B, 2A1C, 2A2, 2B1A, 2B1B, 2B2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -4945,6 +5330,11 @@
           <t>461</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -4952,6 +5342,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -4959,6 +5354,11 @@
           <t>463</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -4966,6 +5366,11 @@
           <t>464A</t>
         </is>
       </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -4973,6 +5378,11 @@
           <t>464B</t>
         </is>
       </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A2C, 1A3, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -4980,6 +5390,11 @@
           <t>465A</t>
         </is>
       </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B1, 2B2, 2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -4987,6 +5402,11 @@
           <t>465B</t>
         </is>
       </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1, 1A2, 1A3, 1B, 2, 3A, 3B1, 3B1B, 3B2, 4A1, 4A2, 4B, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -4994,6 +5414,11 @@
           <t>466</t>
         </is>
       </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -5001,6 +5426,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -5008,6 +5438,11 @@
           <t>468A</t>
         </is>
       </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -5015,6 +5450,11 @@
           <t>468B</t>
         </is>
       </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2B, 2B1, 2B2, 3, 4A, 4B, 4C, 5</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -5022,11 +5462,21 @@
           <t>469</t>
         </is>
       </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
           <t>47</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 2A, 2B1, 2B2, 2C</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 55 village workbooks (randomwalk-TRX50-WS 2026-10-10T04:49:09Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -5486,6 +5486,11 @@
           <t>470</t>
         </is>
       </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -5493,6 +5498,11 @@
           <t>471</t>
         </is>
       </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2A1, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -5500,6 +5510,11 @@
           <t>472</t>
         </is>
       </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -5507,6 +5522,11 @@
           <t>473</t>
         </is>
       </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -5514,6 +5534,11 @@
           <t>474</t>
         </is>
       </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -5521,6 +5546,11 @@
           <t>475</t>
         </is>
       </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -5528,6 +5558,11 @@
           <t>476</t>
         </is>
       </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -5535,6 +5570,11 @@
           <t>477</t>
         </is>
       </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -5542,6 +5582,11 @@
           <t>478</t>
         </is>
       </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -5549,6 +5594,11 @@
           <t>479</t>
         </is>
       </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -5556,6 +5606,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -5563,6 +5618,11 @@
           <t>480</t>
         </is>
       </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -5570,6 +5630,11 @@
           <t>481</t>
         </is>
       </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -5577,6 +5642,11 @@
           <t>482</t>
         </is>
       </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1A, 2B1B, 2B1C, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -5584,6 +5654,11 @@
           <t>483</t>
         </is>
       </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -5591,6 +5666,11 @@
           <t>484</t>
         </is>
       </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -5598,6 +5678,11 @@
           <t>485</t>
         </is>
       </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -5605,6 +5690,11 @@
           <t>486</t>
         </is>
       </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A1C, 1A1D, 1A2, 1A3, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -5612,6 +5702,11 @@
           <t>487</t>
         </is>
       </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -5619,6 +5714,11 @@
           <t>488</t>
         </is>
       </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -5626,6 +5726,11 @@
           <t>489</t>
         </is>
       </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -5633,6 +5738,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -5640,6 +5750,11 @@
           <t>490</t>
         </is>
       </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E1, 1E2, 2A, 2B, 2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -5647,6 +5762,11 @@
           <t>491</t>
         </is>
       </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -5654,6 +5774,11 @@
           <t>492</t>
         </is>
       </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -5661,6 +5786,11 @@
           <t>493</t>
         </is>
       </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -5668,6 +5798,11 @@
           <t>494</t>
         </is>
       </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -5675,6 +5810,11 @@
           <t>495</t>
         </is>
       </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -5682,6 +5822,11 @@
           <t>496</t>
         </is>
       </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -5689,6 +5834,11 @@
           <t>497</t>
         </is>
       </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -5696,6 +5846,11 @@
           <t>498</t>
         </is>
       </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -5703,6 +5858,11 @@
           <t>499</t>
         </is>
       </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -5710,6 +5870,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 2B4, 3A, 3B1A, 3B1B, 3B1C, 3B2, 3B3, 3B4, 4</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -5717,6 +5882,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -5724,6 +5894,11 @@
           <t>501</t>
         </is>
       </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2, 3A, 3B1, 3B2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -5731,6 +5906,11 @@
           <t>502</t>
         </is>
       </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -5738,6 +5918,11 @@
           <t>503</t>
         </is>
       </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -5745,6 +5930,11 @@
           <t>504</t>
         </is>
       </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -5752,6 +5942,11 @@
           <t>505</t>
         </is>
       </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -5759,6 +5954,11 @@
           <t>506</t>
         </is>
       </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -5766,6 +5966,11 @@
           <t>507</t>
         </is>
       </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3A1, 2A3A2, 2A3B, 2B, 3, 4A, 4B1, 4B2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -5773,6 +5978,11 @@
           <t>508</t>
         </is>
       </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -5780,6 +5990,11 @@
           <t>509</t>
         </is>
       </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -5787,6 +6002,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A1A1A, 1A1B, 1A2, 1A3, 1B1, 1B2, 2A1A, 2A1B, 2A1C, 2A2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -5794,6 +6014,11 @@
           <t>510</t>
         </is>
       </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -5801,6 +6026,11 @@
           <t>511</t>
         </is>
       </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -5808,6 +6038,11 @@
           <t>512</t>
         </is>
       </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -5815,6 +6050,11 @@
           <t>513</t>
         </is>
       </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -5822,6 +6062,11 @@
           <t>514</t>
         </is>
       </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -5829,6 +6074,11 @@
           <t>515</t>
         </is>
       </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -5836,6 +6086,11 @@
           <t>516</t>
         </is>
       </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -5843,6 +6098,11 @@
           <t>517</t>
         </is>
       </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -5850,6 +6110,11 @@
           <t>518</t>
         </is>
       </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -5857,6 +6122,11 @@
           <t>519</t>
         </is>
       </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -5864,6 +6134,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -5871,6 +6146,11 @@
           <t>520</t>
         </is>
       </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -5878,6 +6158,11 @@
           <t>521</t>
         </is>
       </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A2, 1A3, 1B, 2, 3A, 3B, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -5885,6 +6170,11 @@
           <t>522</t>
         </is>
       </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -5892,6 +6182,11 @@
           <t>523A</t>
         </is>
       </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -5899,6 +6194,11 @@
           <t>523B</t>
         </is>
       </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -5906,6 +6206,11 @@
           <t>523C</t>
         </is>
       </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -5913,6 +6218,11 @@
           <t>524A</t>
         </is>
       </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1A2C1, 1A2C2, 1A2C3</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -5920,6 +6230,11 @@
           <t>524B</t>
         </is>
       </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B1C, 1B2A, 1B2B, 1B2C</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -5927,6 +6242,11 @@
           <t>525</t>
         </is>
       </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -5934,6 +6254,11 @@
           <t>526</t>
         </is>
       </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -5941,6 +6266,11 @@
           <t>527</t>
         </is>
       </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -5948,6 +6278,11 @@
           <t>528</t>
         </is>
       </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -5955,6 +6290,11 @@
           <t>529A</t>
         </is>
       </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 2C1, 2C2, 2C3</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -5962,6 +6302,11 @@
           <t>529B</t>
         </is>
       </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -5969,6 +6314,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -5976,6 +6326,11 @@
           <t>530A</t>
         </is>
       </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -5983,6 +6338,11 @@
           <t>530B</t>
         </is>
       </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -5990,6 +6350,11 @@
           <t>531</t>
         </is>
       </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -5997,6 +6362,11 @@
           <t>532</t>
         </is>
       </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A1D, 1A1E, 1A1F, 1A2, 1B, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -6004,6 +6374,11 @@
           <t>533</t>
         </is>
       </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -6011,6 +6386,11 @@
           <t>534</t>
         </is>
       </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>10, 1A, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -6018,6 +6398,11 @@
           <t>535</t>
         </is>
       </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -6025,6 +6410,11 @@
           <t>536</t>
         </is>
       </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B1A, 2B1B, 2B2, 2B3A, 2B3B, 2B3C1, 2B3C2, 2B3D</t>
+        </is>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -6032,6 +6422,11 @@
           <t>537</t>
         </is>
       </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -6039,6 +6434,11 @@
           <t>538</t>
         </is>
       </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -6046,6 +6446,11 @@
           <t>539</t>
         </is>
       </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -6053,11 +6458,21 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2A1, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
           <t>540</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 55 village workbooks (randomwalk-TRX50-WS 2026-10-10T09:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -6482,6 +6482,11 @@
           <t>541</t>
         </is>
       </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -6489,6 +6494,11 @@
           <t>542</t>
         </is>
       </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -6496,6 +6506,11 @@
           <t>543</t>
         </is>
       </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A1, 4A2, 4B, 4C, 4D, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -6503,6 +6518,11 @@
           <t>544</t>
         </is>
       </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -6510,6 +6530,11 @@
           <t>545</t>
         </is>
       </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B1, 2B2, 2C, 2D, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -6517,6 +6542,11 @@
           <t>546</t>
         </is>
       </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2A, 1B2B, 2A1, 2A2, 2B1, 2B2, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -6524,6 +6554,11 @@
           <t>547</t>
         </is>
       </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -6531,6 +6566,11 @@
           <t>548</t>
         </is>
       </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -6538,6 +6578,11 @@
           <t>549</t>
         </is>
       </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B, 7A, 7B1, 7B2</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -6545,6 +6590,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -6552,6 +6602,11 @@
           <t>550</t>
         </is>
       </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -6559,6 +6614,11 @@
           <t>551</t>
         </is>
       </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -6566,6 +6626,11 @@
           <t>552</t>
         </is>
       </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -6573,6 +6638,11 @@
           <t>553</t>
         </is>
       </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B1, 3C1A1, 3C1A2, 3C1B1, 3C1B2, 3C1B3, 3C2, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -6580,6 +6650,11 @@
           <t>554</t>
         </is>
       </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -6587,6 +6662,11 @@
           <t>555</t>
         </is>
       </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -6594,6 +6674,11 @@
           <t>556</t>
         </is>
       </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
@@ -6601,6 +6686,11 @@
           <t>557</t>
         </is>
       </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B1, 3B2, 3B3, 4A1, 4A2, 4A3, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -6608,6 +6698,11 @@
           <t>558</t>
         </is>
       </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -6615,6 +6710,11 @@
           <t>559</t>
         </is>
       </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -6622,6 +6722,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4A1A1, 4A1A2, 4A1A3, 4A1A4, 4A1B, 4A2, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -6629,6 +6734,11 @@
           <t>560</t>
         </is>
       </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -6636,6 +6746,11 @@
           <t>561</t>
         </is>
       </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
@@ -6643,6 +6758,11 @@
           <t>562</t>
         </is>
       </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -6650,6 +6770,11 @@
           <t>563</t>
         </is>
       </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -6657,6 +6782,11 @@
           <t>564</t>
         </is>
       </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -6664,11 +6794,21 @@
           <t>565</t>
         </is>
       </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B1, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
           <t>566</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 55 village workbooks (randomwalk-TRX50-WS 2026-10-10T09:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -6818,6 +6818,11 @@
           <t>567</t>
         </is>
       </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -6825,6 +6830,11 @@
           <t>568</t>
         </is>
       </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -6832,6 +6842,11 @@
           <t>569</t>
         </is>
       </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -6839,6 +6854,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -6846,6 +6866,11 @@
           <t>570</t>
         </is>
       </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -6853,6 +6878,11 @@
           <t>571</t>
         </is>
       </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -6860,6 +6890,11 @@
           <t>572</t>
         </is>
       </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -6867,6 +6902,11 @@
           <t>573</t>
         </is>
       </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -6874,6 +6914,11 @@
           <t>574</t>
         </is>
       </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -6881,6 +6926,11 @@
           <t>575</t>
         </is>
       </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -6888,6 +6938,11 @@
           <t>576</t>
         </is>
       </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -6895,6 +6950,11 @@
           <t>577</t>
         </is>
       </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -6902,6 +6962,11 @@
           <t>578</t>
         </is>
       </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -6909,6 +6974,11 @@
           <t>579</t>
         </is>
       </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -6916,6 +6986,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1A, 1C1B, 1C2, 1D, 1E1A, 1E1B, 1E1C, 1E1D, 1E2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -6923,6 +6998,11 @@
           <t>580</t>
         </is>
       </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -6930,6 +7010,11 @@
           <t>581</t>
         </is>
       </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -6937,6 +7022,11 @@
           <t>582</t>
         </is>
       </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -6944,6 +7034,11 @@
           <t>583</t>
         </is>
       </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -6951,6 +7046,11 @@
           <t>584</t>
         </is>
       </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -6958,6 +7058,11 @@
           <t>585</t>
         </is>
       </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -6965,6 +7070,11 @@
           <t>586</t>
         </is>
       </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -6972,6 +7082,11 @@
           <t>587</t>
         </is>
       </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -6979,6 +7094,11 @@
           <t>588A</t>
         </is>
       </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -6986,6 +7106,11 @@
           <t>588B</t>
         </is>
       </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -6993,6 +7118,11 @@
           <t>589</t>
         </is>
       </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -7000,6 +7130,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -7007,6 +7142,11 @@
           <t>590A</t>
         </is>
       </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -7014,6 +7154,11 @@
           <t>590B</t>
         </is>
       </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -7021,6 +7166,11 @@
           <t>591</t>
         </is>
       </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 2A1, 2A2, 2B, 2C, 2D, 2E, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
@@ -7028,6 +7178,11 @@
           <t>592</t>
         </is>
       </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -7035,6 +7190,11 @@
           <t>593A</t>
         </is>
       </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -7042,6 +7202,11 @@
           <t>593B</t>
         </is>
       </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -7049,6 +7214,11 @@
           <t>594</t>
         </is>
       </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -7056,6 +7226,11 @@
           <t>595A</t>
         </is>
       </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
@@ -7063,6 +7238,11 @@
           <t>595B</t>
         </is>
       </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -7070,6 +7250,11 @@
           <t>595C</t>
         </is>
       </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 6, 7A, 7B, 7C, 7D</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -7077,6 +7262,11 @@
           <t>596</t>
         </is>
       </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -7084,6 +7274,11 @@
           <t>597</t>
         </is>
       </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -7091,6 +7286,11 @@
           <t>598</t>
         </is>
       </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -7098,6 +7298,11 @@
           <t>599</t>
         </is>
       </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A1, 4A2, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -7105,6 +7310,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -7112,6 +7322,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -7119,6 +7334,11 @@
           <t>600</t>
         </is>
       </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -7126,6 +7346,11 @@
           <t>601</t>
         </is>
       </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -7133,6 +7358,11 @@
           <t>602</t>
         </is>
       </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
@@ -7140,6 +7370,11 @@
           <t>603</t>
         </is>
       </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
@@ -7147,6 +7382,11 @@
           <t>604</t>
         </is>
       </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C1, 1A1C2, 1A2, 1A3, 1A4, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
@@ -7154,6 +7394,11 @@
           <t>605</t>
         </is>
       </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
@@ -7161,6 +7406,11 @@
           <t>606</t>
         </is>
       </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5A, 1A5B, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -7168,6 +7418,11 @@
           <t>607</t>
         </is>
       </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -7175,6 +7430,11 @@
           <t>608</t>
         </is>
       </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B1, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
@@ -7182,6 +7442,11 @@
           <t>609</t>
         </is>
       </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
@@ -7189,6 +7454,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
@@ -7196,6 +7466,11 @@
           <t>610</t>
         </is>
       </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
@@ -7203,6 +7478,11 @@
           <t>611</t>
         </is>
       </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -7210,6 +7490,11 @@
           <t>612</t>
         </is>
       </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1, 1D2, 1E1A, 1E1B, 1E2, 1F1A, 1F2, 2A1A1, 2A2, 2B, 3, 4, 5, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
@@ -7217,6 +7502,11 @@
           <t>613</t>
         </is>
       </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -7224,6 +7514,11 @@
           <t>614</t>
         </is>
       </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -7231,6 +7526,11 @@
           <t>615</t>
         </is>
       </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -7238,6 +7538,11 @@
           <t>616</t>
         </is>
       </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
@@ -7245,6 +7550,11 @@
           <t>617</t>
         </is>
       </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
@@ -7252,6 +7562,11 @@
           <t>618</t>
         </is>
       </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
@@ -7259,6 +7574,11 @@
           <t>619</t>
         </is>
       </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
@@ -7266,6 +7586,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -7273,6 +7598,11 @@
           <t>620</t>
         </is>
       </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -7280,6 +7610,11 @@
           <t>621</t>
         </is>
       </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
@@ -7287,6 +7622,11 @@
           <t>622</t>
         </is>
       </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1A, 2B2, 2B3, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -7294,6 +7634,11 @@
           <t>623</t>
         </is>
       </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
@@ -7301,6 +7646,11 @@
           <t>624</t>
         </is>
       </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -7308,11 +7658,21 @@
           <t>625</t>
         </is>
       </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
           <t>626</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 56 village workbooks (sivaramans-llin 2026-10-10T14:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -7682,6 +7682,11 @@
           <t>627</t>
         </is>
       </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -7689,6 +7694,11 @@
           <t>628</t>
         </is>
       </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -7696,6 +7706,11 @@
           <t>629</t>
         </is>
       </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B1, 5B2, 6</t>
+        </is>
+      </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
@@ -7703,6 +7718,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -7710,6 +7730,11 @@
           <t>630</t>
         </is>
       </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2A1, 2A2, 2B1, 2B2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -7717,6 +7742,11 @@
           <t>631</t>
         </is>
       </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -7724,6 +7754,11 @@
           <t>632</t>
         </is>
       </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -7731,6 +7766,11 @@
           <t>633</t>
         </is>
       </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -7738,6 +7778,11 @@
           <t>634</t>
         </is>
       </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -7745,6 +7790,11 @@
           <t>635</t>
         </is>
       </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
@@ -7752,6 +7802,11 @@
           <t>636</t>
         </is>
       </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -7759,6 +7814,11 @@
           <t>637</t>
         </is>
       </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -7766,6 +7826,11 @@
           <t>638</t>
         </is>
       </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -7773,6 +7838,11 @@
           <t>639</t>
         </is>
       </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -7780,6 +7850,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1A2C, 1B, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -7787,6 +7862,11 @@
           <t>640</t>
         </is>
       </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
@@ -7794,6 +7874,11 @@
           <t>641</t>
         </is>
       </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -7801,6 +7886,11 @@
           <t>642</t>
         </is>
       </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
@@ -7808,6 +7898,11 @@
           <t>643</t>
         </is>
       </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -7815,6 +7910,11 @@
           <t>644</t>
         </is>
       </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -7822,6 +7922,11 @@
           <t>645</t>
         </is>
       </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -7829,6 +7934,11 @@
           <t>646</t>
         </is>
       </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
@@ -7836,6 +7946,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 2C, 2D, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
@@ -7843,6 +7958,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
@@ -7850,6 +7970,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
@@ -7857,6 +7982,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2, 1A3, 1A4, 1B, 1C, 1D, 1E, 1F, 1G, 2A1, 2A2, 2B1, 2B2, 2B3, 2B4, 2B5, 3A1A1, 3A1A2, 3A1B, 3A1C1, 3A1C2, 3A2, 3B1A1, 3B1B, 3B2, 3B3, 4A1A, 4A1B, 4A2, 4B1, 4B2, 4B3, 5</t>
+        </is>
+      </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
@@ -7864,6 +7994,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -7871,6 +8006,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -7878,6 +8018,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -7885,6 +8030,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B1A, 3B1B, 3B2A, 3B2B, 3B2C</t>
+        </is>
+      </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
@@ -7892,6 +8042,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -7899,6 +8054,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20A, 20B, 21A, 21B, 21C, 22A, 22B, 22C, 3, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 6A1, 6A2, 6B, 6C, 7, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -7906,6 +8066,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B1, 1B2, 2A1, 2A2A, 2A2B, 2B1, 2B2, 2C, 2D, 2E, 3, 4A, 4B, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -7913,6 +8078,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A1A1A1, 1A1B, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1B1A, 1B2, 1C, 1D1, 1D2, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -7920,6 +8090,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1A1A1, 1C1B, 1C1C, 1C2, 1C3, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -7927,6 +8102,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1B, 1A2, 1A3, 1B1A1A, 1B1B, 1B2, 1B3, 2A1, 2A2, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
@@ -7934,6 +8114,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
@@ -7941,6 +8126,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
@@ -7948,11 +8138,21 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
           <t>80</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1, 1A1A2, 1A1A3, 1A1B1, 1A1B2, 1A2A1, 1B1, 1B2, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 57 village workbooks (sivaramans-llin 2026-10-10T14:38:40Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Athupakkam_13.427855_80.150297.xlsx
@@ -8162,6 +8162,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A1A, 5A1B, 5A2, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
@@ -8169,6 +8174,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3A1A, 3A1B, 3A2, 3B1, 3B2A, 3B2B, 3B3, 3B4, 3C1, 3C2, 4A1, 4A2, 4B, 5A, 5B, 6A, 6B, 6C, 6D, 6E1, 6E2, 7A, 7B, 7C, 8</t>
+        </is>
+      </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
@@ -8176,6 +8186,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B1, 1B2, 1C, 2A1A, 2A1B, 2A1C, 2A2A1, 2A2A2, 2A2B, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -8183,6 +8198,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
@@ -8190,6 +8210,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -8197,6 +8222,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -8204,6 +8234,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4, 5, 6A, 6B, 7A, 7B1, 7B2</t>
+        </is>
+      </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
@@ -8211,6 +8246,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 3A, 3B1, 3B2, 4A, 4B, 5, 6A, 6B, 6C, 7A, 7B1, 7B2, 7C1A, 7C1B, 7C2, 7D</t>
+        </is>
+      </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
@@ -8218,6 +8258,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -8225,6 +8270,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1C, 1D, 1E, 2, 3A, 3B, 4A, 4B, 4C, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
@@ -8232,6 +8282,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B1, 3B2, 4A1, 4A2A, 4A2B, 4A2C, 4B1, 4B2, 4B3A, 5</t>
+        </is>
+      </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
@@ -8239,6 +8294,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
@@ -8246,6 +8306,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 3A1, 3A2, 3B, 3C, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
@@ -8253,6 +8318,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 3A, 3B, 4A, 4B, 4C, 5A, 5B, 5C, 5D, 5E, 5F, 5G</t>
+        </is>
+      </c>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
@@ -8260,6 +8330,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -8267,6 +8342,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
@@ -8274,11 +8354,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>